<commit_message>
docs: finalize QA portfolio presentation
</commit_message>
<xml_diff>
--- a/01-ecommerce-qa-case-study/test-cases/04-live-test-execution.xlsx
+++ b/01-ecommerce-qa-case-study/test-cases/04-live-test-execution.xlsx
@@ -753,7 +753,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="N3" s="29" t="str">
-        <x:v>evidence/execution/auth/EXEC-TC-AUTH-002.png</x:v>
+        <x:v>No supporting screenshot retained; see Actual Result.</x:v>
       </x:c>
       <x:c r="O3" s="23" t="str">
         <x:v>Confirm the account still exists before execution.
@@ -807,7 +807,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="N4" s="29" t="str">
-        <x:v>evidence/execution/auth/EXEC-TC-AUTH-003.png</x:v>
+        <x:v>evidence/discovery/auth/AUTH-EV-004.png</x:v>
       </x:c>
       <x:c r="O4" s="23" t="str">
         <x:v>Single invalid attempt only; no lockout or throttling checks.
@@ -1128,7 +1128,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="N10" s="29" t="str">
-        <x:v>evidence/execution/discovery/EXEC-TC-DISC-005.png</x:v>
+        <x:v>evidence/discovery/discovery/DISC-EV-NIKE.png</x:v>
       </x:c>
       <x:c r="O10" s="23" t="str">
         <x:v>Do not combine multiple filters or test price sliders.
@@ -1503,7 +1503,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="N17" s="29" t="str">
-        <x:v>evidence/execution/cart/EXEC-TC-CART-003.png</x:v>
+        <x:v>evidence/discovery/cart/CART-EV-004.png</x:v>
       </x:c>
       <x:c r="O17" s="23" t="str">
         <x:v>Bounded to final-item removal.
@@ -1558,7 +1558,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="N18" s="29" t="str">
-        <x:v>evidence/execution/cart/EXEC-TC-CART-004.png</x:v>
+        <x:v>No supporting screenshot retained; see Actual Result.</x:v>
       </x:c>
       <x:c r="O18" s="23" t="str">
         <x:v>Guest-cart merging after authentication is outside scope.
@@ -1613,7 +1613,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="N19" s="29" t="str">
-        <x:v>evidence/execution/cart/EXEC-TC-CART-005.png</x:v>
+        <x:v>No supporting screenshot retained; see Actual Result.</x:v>
       </x:c>
       <x:c r="O19" s="23" t="str">
         <x:v>Configuration must match exactly.
@@ -1834,7 +1834,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="N23" s="29" t="str">
-        <x:v>evidence/execution/checkout/EXEC-TC-CHK-003.png</x:v>
+        <x:v>evidence/discovery/checkout/CHK-EV-004.png</x:v>
       </x:c>
       <x:c r="O23" s="23" t="str">
         <x:v>Credit-card authorization and processing are outside scope.
@@ -1887,7 +1887,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="N24" s="29" t="str">
-        <x:v>evidence/execution/checkout/EXEC-TC-CHK-004.png</x:v>
+        <x:v>evidence/discovery/checkout/CHK-EV-005.png</x:v>
       </x:c>
       <x:c r="O24" s="23" t="str">
         <x:v>Do not use real payment credentials.
@@ -1940,7 +1940,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="N25" s="30" t="str">
-        <x:v>evidence/execution/checkout/EXEC-TC-CHK-005.png</x:v>
+        <x:v>evidence/discovery/cart/CART-EV-004.png</x:v>
       </x:c>
       <x:c r="O25" s="24" t="str">
         <x:v>Execute immediately after TC-CHK-004 in the same session.

</xml_diff>